<commit_message>
mise a jour des modèles
</commit_message>
<xml_diff>
--- a/liste des station.xlsx
+++ b/liste des station.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bpsabj-my.sharepoint.com/personal/gganye_beninpetro_com/Documents/Documents/Projet_prediction/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bpsabj-my.sharepoint.com/personal/gganye_beninpetro_com/Documents/Documents/memoire_bi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="752" documentId="8_{245ECF86-76A3-4D04-817D-C5456EB42609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C61B35A7-1BF8-4647-88A1-91319DDFA70D}"/>
+  <xr:revisionPtr revIDLastSave="761" documentId="8_{245ECF86-76A3-4D04-817D-C5456EB42609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{67E15CA2-50A0-41EF-9CF6-7D1B55CA3C83}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{7A6CA190-2837-4F4B-BF5A-6119A87CF2E8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{7A6CA190-2837-4F4B-BF5A-6119A87CF2E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -1597,7 +1597,7 @@
     <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1616,7 +1616,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Milliers [0]" xfId="1" builtinId="6"/>
@@ -1624,13 +1623,6 @@
     <cellStyle name="Normal 2" xfId="2" xr:uid="{EA9C4F65-BC71-4D7D-BEAE-96C29653BFC8}"/>
   </cellStyles>
   <dxfs count="24">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -1768,6 +1760,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1951,7 +1950,7 @@
     <tableColumn id="1" xr3:uid="{D4006DC3-467C-4753-931B-20D153A6C562}" name="Code Station" dataDxfId="15">
       <calculatedColumnFormula array="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D2,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D2,$D$2:$D$148,0)-1)))),"0000")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{E8A8DF2A-258C-4161-8EDE-1E58C6262F3E}" name="GROUPE TYPE" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{E8A8DF2A-258C-4161-8EDE-1E58C6262F3E}" name="GROUPE TYPE" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2335,7 +2334,7 @@
         <f t="array" aca="1" ref="G2" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D2,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D2,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0001</v>
       </c>
-      <c r="H2" s="8" t="s">
+      <c r="H2" t="s">
         <v>483</v>
       </c>
     </row>
@@ -2362,7 +2361,7 @@
         <f t="array" aca="1" ref="G3" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D3,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D3,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0002</v>
       </c>
-      <c r="H3" s="8" t="str">
+      <c r="H3" t="str">
         <f>H2</f>
         <v>STATION</v>
       </c>
@@ -2390,7 +2389,7 @@
         <f t="array" aca="1" ref="G4" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D4,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D4,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0003</v>
       </c>
-      <c r="H4" s="8" t="str">
+      <c r="H4" t="str">
         <f t="shared" ref="H4:H67" si="0">H3</f>
         <v>STATION</v>
       </c>
@@ -2418,7 +2417,7 @@
         <f t="array" aca="1" ref="G5" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D5,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D5,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0004</v>
       </c>
-      <c r="H5" s="8" t="str">
+      <c r="H5" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2446,7 +2445,7 @@
         <f t="array" aca="1" ref="G6" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D6,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D6,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0004</v>
       </c>
-      <c r="H6" s="8" t="str">
+      <c r="H6" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2474,7 +2473,7 @@
         <f t="array" aca="1" ref="G7" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D7,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D7,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0005</v>
       </c>
-      <c r="H7" s="8" t="str">
+      <c r="H7" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2502,7 +2501,7 @@
         <f t="array" aca="1" ref="G8" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D8,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D8,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0006</v>
       </c>
-      <c r="H8" s="8" t="str">
+      <c r="H8" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2530,7 +2529,7 @@
         <f t="array" aca="1" ref="G9" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D9,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D9,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0007</v>
       </c>
-      <c r="H9" s="8" t="str">
+      <c r="H9" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2558,7 +2557,7 @@
         <f t="array" aca="1" ref="G10" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D10,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D10,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0008</v>
       </c>
-      <c r="H10" s="8" t="str">
+      <c r="H10" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2586,7 +2585,7 @@
         <f t="array" aca="1" ref="G11" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D11,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D11,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0009</v>
       </c>
-      <c r="H11" s="8" t="str">
+      <c r="H11" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2614,7 +2613,7 @@
         <f t="array" aca="1" ref="G12" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D12,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D12,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0010</v>
       </c>
-      <c r="H12" s="8" t="str">
+      <c r="H12" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2642,7 +2641,7 @@
         <f t="array" aca="1" ref="G13" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D13,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D13,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0011</v>
       </c>
-      <c r="H13" s="8" t="str">
+      <c r="H13" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2670,7 +2669,7 @@
         <f t="array" aca="1" ref="G14" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D14,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D14,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0012</v>
       </c>
-      <c r="H14" s="8" t="str">
+      <c r="H14" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2698,7 +2697,7 @@
         <f t="array" aca="1" ref="G15" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D15,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D15,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0013</v>
       </c>
-      <c r="H15" s="8" t="str">
+      <c r="H15" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2726,7 +2725,7 @@
         <f t="array" aca="1" ref="G16" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D16,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D16,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0014</v>
       </c>
-      <c r="H16" s="8" t="str">
+      <c r="H16" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2754,7 +2753,7 @@
         <f t="array" aca="1" ref="G17" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D17,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D17,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0015</v>
       </c>
-      <c r="H17" s="8" t="str">
+      <c r="H17" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2782,7 +2781,7 @@
         <f t="array" aca="1" ref="G18" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D18,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D18,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0016</v>
       </c>
-      <c r="H18" s="8" t="str">
+      <c r="H18" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2810,7 +2809,7 @@
         <f t="array" aca="1" ref="G19" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D19,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D19,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0017</v>
       </c>
-      <c r="H19" s="8" t="str">
+      <c r="H19" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2838,7 +2837,7 @@
         <f t="array" aca="1" ref="G20" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D20,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D20,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0018</v>
       </c>
-      <c r="H20" s="8" t="str">
+      <c r="H20" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2866,7 +2865,7 @@
         <f t="array" aca="1" ref="G21" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D21,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D21,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0019</v>
       </c>
-      <c r="H21" s="8" t="str">
+      <c r="H21" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2894,7 +2893,7 @@
         <f t="array" aca="1" ref="G22" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D22,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D22,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0020</v>
       </c>
-      <c r="H22" s="8" t="str">
+      <c r="H22" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2922,7 +2921,7 @@
         <f t="array" aca="1" ref="G23" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D23,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D23,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0018</v>
       </c>
-      <c r="H23" s="8" t="str">
+      <c r="H23" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2950,7 +2949,7 @@
         <f t="array" aca="1" ref="G24" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D24,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D24,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0021</v>
       </c>
-      <c r="H24" s="8" t="str">
+      <c r="H24" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -2978,7 +2977,7 @@
         <f t="array" aca="1" ref="G25" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D25,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D25,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0017</v>
       </c>
-      <c r="H25" s="8" t="str">
+      <c r="H25" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3006,7 +3005,7 @@
         <f t="array" aca="1" ref="G26" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D26,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D26,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0022</v>
       </c>
-      <c r="H26" s="8" t="str">
+      <c r="H26" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3034,7 +3033,7 @@
         <f t="array" aca="1" ref="G27" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D27,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D27,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0023</v>
       </c>
-      <c r="H27" s="8" t="str">
+      <c r="H27" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3062,7 +3061,7 @@
         <f t="array" aca="1" ref="G28" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D28,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D28,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0024</v>
       </c>
-      <c r="H28" s="8" t="str">
+      <c r="H28" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3090,7 +3089,7 @@
         <f t="array" aca="1" ref="G29" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D29,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D29,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0015</v>
       </c>
-      <c r="H29" s="8" t="str">
+      <c r="H29" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3118,7 +3117,7 @@
         <f t="array" aca="1" ref="G30" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D30,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D30,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0025</v>
       </c>
-      <c r="H30" s="8" t="str">
+      <c r="H30" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3146,7 +3145,7 @@
         <f t="array" aca="1" ref="G31" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D31,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D31,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0026</v>
       </c>
-      <c r="H31" s="8" t="str">
+      <c r="H31" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3174,7 +3173,7 @@
         <f t="array" aca="1" ref="G32" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D32,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D32,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0027</v>
       </c>
-      <c r="H32" s="8" t="str">
+      <c r="H32" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3202,7 +3201,7 @@
         <f t="array" aca="1" ref="G33" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D33,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D33,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0010</v>
       </c>
-      <c r="H33" s="8" t="str">
+      <c r="H33" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3230,7 +3229,7 @@
         <f t="array" aca="1" ref="G34" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D34,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D34,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0020</v>
       </c>
-      <c r="H34" s="8" t="str">
+      <c r="H34" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3258,7 +3257,7 @@
         <f t="array" aca="1" ref="G35" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D35,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D35,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0028</v>
       </c>
-      <c r="H35" s="8" t="str">
+      <c r="H35" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3286,7 +3285,7 @@
         <f t="array" aca="1" ref="G36" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D36,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D36,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0026</v>
       </c>
-      <c r="H36" s="8" t="str">
+      <c r="H36" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3314,7 +3313,7 @@
         <f t="array" aca="1" ref="G37" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D37,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D37,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0029</v>
       </c>
-      <c r="H37" s="8" t="str">
+      <c r="H37" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3342,7 +3341,7 @@
         <f t="array" aca="1" ref="G38" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D38,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D38,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0030</v>
       </c>
-      <c r="H38" s="8" t="str">
+      <c r="H38" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3370,7 +3369,7 @@
         <f t="array" aca="1" ref="G39" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D39,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D39,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0031</v>
       </c>
-      <c r="H39" s="8" t="str">
+      <c r="H39" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3398,7 +3397,7 @@
         <f t="array" aca="1" ref="G40" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D40,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D40,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0032</v>
       </c>
-      <c r="H40" s="8" t="str">
+      <c r="H40" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3426,7 +3425,7 @@
         <f t="array" aca="1" ref="G41" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D41,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D41,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0033</v>
       </c>
-      <c r="H41" s="8" t="str">
+      <c r="H41" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3454,7 +3453,7 @@
         <f t="array" aca="1" ref="G42" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D42,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D42,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0034</v>
       </c>
-      <c r="H42" s="8" t="str">
+      <c r="H42" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3482,7 +3481,7 @@
         <f t="array" aca="1" ref="G43" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D43,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D43,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0035</v>
       </c>
-      <c r="H43" s="8" t="str">
+      <c r="H43" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3510,7 +3509,7 @@
         <f t="array" aca="1" ref="G44" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D44,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D44,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0036</v>
       </c>
-      <c r="H44" s="8" t="str">
+      <c r="H44" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3538,7 +3537,7 @@
         <f t="array" aca="1" ref="G45" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D45,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D45,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0037</v>
       </c>
-      <c r="H45" s="8" t="str">
+      <c r="H45" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3566,7 +3565,7 @@
         <f t="array" aca="1" ref="G46" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D46,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D46,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0038</v>
       </c>
-      <c r="H46" s="8" t="str">
+      <c r="H46" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3594,7 +3593,7 @@
         <f t="array" aca="1" ref="G47" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D47,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D47,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0039</v>
       </c>
-      <c r="H47" s="8" t="str">
+      <c r="H47" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3622,7 +3621,7 @@
         <f t="array" aca="1" ref="G48" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D48,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D48,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0033</v>
       </c>
-      <c r="H48" s="8" t="str">
+      <c r="H48" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3650,7 +3649,7 @@
         <f t="array" aca="1" ref="G49" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D49,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D49,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0040</v>
       </c>
-      <c r="H49" s="8" t="str">
+      <c r="H49" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3678,7 +3677,7 @@
         <f t="array" aca="1" ref="G50" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D50,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D50,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0041</v>
       </c>
-      <c r="H50" s="8" t="str">
+      <c r="H50" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3706,7 +3705,7 @@
         <f t="array" aca="1" ref="G51" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D51,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D51,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0042</v>
       </c>
-      <c r="H51" s="8" t="str">
+      <c r="H51" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3734,7 +3733,7 @@
         <f t="array" aca="1" ref="G52" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D52,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D52,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0043</v>
       </c>
-      <c r="H52" s="8" t="str">
+      <c r="H52" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3762,7 +3761,7 @@
         <f t="array" aca="1" ref="G53" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D53,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D53,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0044</v>
       </c>
-      <c r="H53" s="8" t="str">
+      <c r="H53" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3790,7 +3789,7 @@
         <f t="array" aca="1" ref="G54" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D54,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D54,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0045</v>
       </c>
-      <c r="H54" s="8" t="str">
+      <c r="H54" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3818,7 +3817,7 @@
         <f t="array" aca="1" ref="G55" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D55,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D55,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0045</v>
       </c>
-      <c r="H55" s="8" t="str">
+      <c r="H55" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3846,7 +3845,7 @@
         <f t="array" aca="1" ref="G56" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D56,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D56,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0046</v>
       </c>
-      <c r="H56" s="8" t="str">
+      <c r="H56" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3874,7 +3873,7 @@
         <f t="array" aca="1" ref="G57" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D57,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D57,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0024</v>
       </c>
-      <c r="H57" s="8" t="str">
+      <c r="H57" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3902,7 +3901,7 @@
         <f t="array" aca="1" ref="G58" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D58,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D58,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0047</v>
       </c>
-      <c r="H58" s="8" t="str">
+      <c r="H58" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3930,7 +3929,7 @@
         <f t="array" aca="1" ref="G59" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D59,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D59,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0048</v>
       </c>
-      <c r="H59" s="8" t="str">
+      <c r="H59" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3958,7 +3957,7 @@
         <f t="array" aca="1" ref="G60" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D60,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D60,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0049</v>
       </c>
-      <c r="H60" s="8" t="str">
+      <c r="H60" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -3986,7 +3985,7 @@
         <f t="array" aca="1" ref="G61" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D61,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D61,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0050</v>
       </c>
-      <c r="H61" s="8" t="str">
+      <c r="H61" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4014,7 +4013,7 @@
         <f t="array" aca="1" ref="G62" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D62,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D62,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0051</v>
       </c>
-      <c r="H62" s="8" t="str">
+      <c r="H62" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4042,7 +4041,7 @@
         <f t="array" aca="1" ref="G63" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D63,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D63,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0052</v>
       </c>
-      <c r="H63" s="8" t="str">
+      <c r="H63" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4070,7 +4069,7 @@
         <f t="array" aca="1" ref="G64" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D64,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D64,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0053</v>
       </c>
-      <c r="H64" s="8" t="str">
+      <c r="H64" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4098,7 +4097,7 @@
         <f t="array" aca="1" ref="G65" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D65,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D65,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0054</v>
       </c>
-      <c r="H65" s="8" t="str">
+      <c r="H65" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4126,7 +4125,7 @@
         <f t="array" aca="1" ref="G66" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D66,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D66,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0055</v>
       </c>
-      <c r="H66" s="8" t="str">
+      <c r="H66" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4154,7 +4153,7 @@
         <f t="array" aca="1" ref="G67" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D67,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D67,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0056</v>
       </c>
-      <c r="H67" s="8" t="str">
+      <c r="H67" t="str">
         <f t="shared" si="0"/>
         <v>STATION</v>
       </c>
@@ -4182,7 +4181,7 @@
         <f t="array" aca="1" ref="G68" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D68,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D68,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0039</v>
       </c>
-      <c r="H68" s="8" t="str">
+      <c r="H68" t="str">
         <f t="shared" ref="H68:H131" si="1">H67</f>
         <v>STATION</v>
       </c>
@@ -4210,7 +4209,7 @@
         <f t="array" aca="1" ref="G69" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D69,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D69,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0007</v>
       </c>
-      <c r="H69" s="8" t="str">
+      <c r="H69" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4238,7 +4237,7 @@
         <f t="array" aca="1" ref="G70" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D70,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D70,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0057</v>
       </c>
-      <c r="H70" s="8" t="str">
+      <c r="H70" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4266,7 +4265,7 @@
         <f t="array" aca="1" ref="G71" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D71,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D71,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0058</v>
       </c>
-      <c r="H71" s="8" t="str">
+      <c r="H71" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4294,7 +4293,7 @@
         <f t="array" aca="1" ref="G72" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D72,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D72,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0059</v>
       </c>
-      <c r="H72" s="8" t="str">
+      <c r="H72" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4322,7 +4321,7 @@
         <f t="array" aca="1" ref="G73" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D73,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D73,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0009</v>
       </c>
-      <c r="H73" s="8" t="str">
+      <c r="H73" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4350,7 +4349,7 @@
         <f t="array" aca="1" ref="G74" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D74,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D74,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0014</v>
       </c>
-      <c r="H74" s="8" t="str">
+      <c r="H74" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4378,7 +4377,7 @@
         <f t="array" aca="1" ref="G75" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D75,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D75,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0060</v>
       </c>
-      <c r="H75" s="8" t="str">
+      <c r="H75" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4406,7 +4405,7 @@
         <f t="array" aca="1" ref="G76" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D76,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D76,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0061</v>
       </c>
-      <c r="H76" s="8" t="str">
+      <c r="H76" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4434,7 +4433,7 @@
         <f t="array" aca="1" ref="G77" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D77,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D77,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0024</v>
       </c>
-      <c r="H77" s="8" t="str">
+      <c r="H77" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4462,7 +4461,7 @@
         <f t="array" aca="1" ref="G78" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D78,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D78,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0033</v>
       </c>
-      <c r="H78" s="8" t="str">
+      <c r="H78" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4490,7 +4489,7 @@
         <f t="array" aca="1" ref="G79" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D79,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D79,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0028</v>
       </c>
-      <c r="H79" s="8" t="str">
+      <c r="H79" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4518,7 +4517,7 @@
         <f t="array" aca="1" ref="G80" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D80,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D80,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0062</v>
       </c>
-      <c r="H80" s="8" t="str">
+      <c r="H80" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4546,7 +4545,7 @@
         <f t="array" aca="1" ref="G81" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D81,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D81,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0005</v>
       </c>
-      <c r="H81" s="8" t="str">
+      <c r="H81" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4574,7 +4573,7 @@
         <f t="array" aca="1" ref="G82" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D82,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D82,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0063</v>
       </c>
-      <c r="H82" s="8" t="str">
+      <c r="H82" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4602,7 +4601,7 @@
         <f t="array" aca="1" ref="G83" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D83,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D83,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0064</v>
       </c>
-      <c r="H83" s="8" t="str">
+      <c r="H83" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4630,7 +4629,7 @@
         <f t="array" aca="1" ref="G84" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D84,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D84,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0020</v>
       </c>
-      <c r="H84" s="8" t="str">
+      <c r="H84" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4658,7 +4657,7 @@
         <f t="array" aca="1" ref="G85" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D85,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D85,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0065</v>
       </c>
-      <c r="H85" s="8" t="str">
+      <c r="H85" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4686,7 +4685,7 @@
         <f t="array" aca="1" ref="G86" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D86,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D86,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0014</v>
       </c>
-      <c r="H86" s="8" t="str">
+      <c r="H86" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4714,7 +4713,7 @@
         <f t="array" aca="1" ref="G87" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D87,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D87,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0017</v>
       </c>
-      <c r="H87" s="8" t="str">
+      <c r="H87" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4742,7 +4741,7 @@
         <f t="array" aca="1" ref="G88" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D88,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D88,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0066</v>
       </c>
-      <c r="H88" s="8" t="str">
+      <c r="H88" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4770,7 +4769,7 @@
         <f t="array" aca="1" ref="G89" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D89,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D89,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0018</v>
       </c>
-      <c r="H89" s="8" t="str">
+      <c r="H89" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4798,7 +4797,7 @@
         <f t="array" aca="1" ref="G90" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D90,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D90,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0006</v>
       </c>
-      <c r="H90" s="8" t="str">
+      <c r="H90" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4826,7 +4825,7 @@
         <f t="array" aca="1" ref="G91" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D91,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D91,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0067</v>
       </c>
-      <c r="H91" s="8" t="str">
+      <c r="H91" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4854,7 +4853,7 @@
         <f t="array" aca="1" ref="G92" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D92,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D92,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0068</v>
       </c>
-      <c r="H92" s="8" t="str">
+      <c r="H92" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4882,7 +4881,7 @@
         <f t="array" aca="1" ref="G93" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D93,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D93,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0042</v>
       </c>
-      <c r="H93" s="8" t="str">
+      <c r="H93" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4910,7 +4909,7 @@
         <f t="array" aca="1" ref="G94" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D94,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D94,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0069</v>
       </c>
-      <c r="H94" s="8" t="str">
+      <c r="H94" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4938,7 +4937,7 @@
         <f t="array" aca="1" ref="G95" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D95,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D95,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0070</v>
       </c>
-      <c r="H95" s="8" t="str">
+      <c r="H95" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4966,7 +4965,7 @@
         <f t="array" aca="1" ref="G96" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D96,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D96,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0010</v>
       </c>
-      <c r="H96" s="8" t="str">
+      <c r="H96" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -4994,7 +4993,7 @@
         <f t="array" aca="1" ref="G97" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D97,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D97,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0006</v>
       </c>
-      <c r="H97" s="8" t="str">
+      <c r="H97" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5022,7 +5021,7 @@
         <f t="array" aca="1" ref="G98" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D98,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D98,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0015</v>
       </c>
-      <c r="H98" s="8" t="str">
+      <c r="H98" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5050,7 +5049,7 @@
         <f t="array" aca="1" ref="G99" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D99,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D99,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0022</v>
       </c>
-      <c r="H99" s="8" t="str">
+      <c r="H99" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5078,7 +5077,7 @@
         <f t="array" aca="1" ref="G100" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D100,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D100,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0071</v>
       </c>
-      <c r="H100" s="8" t="str">
+      <c r="H100" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5106,7 +5105,7 @@
         <f t="array" aca="1" ref="G101" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D101,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D101,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0072</v>
       </c>
-      <c r="H101" s="8" t="str">
+      <c r="H101" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5134,7 +5133,7 @@
         <f t="array" aca="1" ref="G102" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D102,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D102,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0073</v>
       </c>
-      <c r="H102" s="8" t="str">
+      <c r="H102" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5162,7 +5161,7 @@
         <f t="array" aca="1" ref="G103" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D103,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D103,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0074</v>
       </c>
-      <c r="H103" s="8" t="str">
+      <c r="H103" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5190,7 +5189,7 @@
         <f t="array" aca="1" ref="G104" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D104,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D104,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0003</v>
       </c>
-      <c r="H104" s="8" t="str">
+      <c r="H104" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5218,7 +5217,7 @@
         <f t="array" aca="1" ref="G105" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D105,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D105,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0075</v>
       </c>
-      <c r="H105" s="8" t="str">
+      <c r="H105" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5246,7 +5245,7 @@
         <f t="array" aca="1" ref="G106" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D106,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D106,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0076</v>
       </c>
-      <c r="H106" s="8" t="str">
+      <c r="H106" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5274,7 +5273,7 @@
         <f t="array" aca="1" ref="G107" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D107,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D107,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0077</v>
       </c>
-      <c r="H107" s="8" t="str">
+      <c r="H107" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5302,7 +5301,7 @@
         <f t="array" aca="1" ref="G108" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D108,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D108,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0058</v>
       </c>
-      <c r="H108" s="8" t="str">
+      <c r="H108" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5330,7 +5329,7 @@
         <f t="array" aca="1" ref="G109" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D109,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D109,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0023</v>
       </c>
-      <c r="H109" s="8" t="str">
+      <c r="H109" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5358,7 +5357,7 @@
         <f t="array" aca="1" ref="G110" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D110,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D110,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0078</v>
       </c>
-      <c r="H110" s="8" t="str">
+      <c r="H110" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5386,7 +5385,7 @@
         <f t="array" aca="1" ref="G111" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D111,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D111,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0079</v>
       </c>
-      <c r="H111" s="8" t="str">
+      <c r="H111" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5414,7 +5413,7 @@
         <f t="array" aca="1" ref="G112" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D112,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D112,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0079</v>
       </c>
-      <c r="H112" s="8" t="str">
+      <c r="H112" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5442,7 +5441,7 @@
         <f t="array" aca="1" ref="G113" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D113,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D113,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0080</v>
       </c>
-      <c r="H113" s="8" t="str">
+      <c r="H113" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5470,7 +5469,7 @@
         <f t="array" aca="1" ref="G114" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D114,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D114,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0081</v>
       </c>
-      <c r="H114" s="8" t="str">
+      <c r="H114" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5498,7 +5497,7 @@
         <f t="array" aca="1" ref="G115" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D115,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D115,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0081</v>
       </c>
-      <c r="H115" s="8" t="str">
+      <c r="H115" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5526,7 +5525,7 @@
         <f t="array" aca="1" ref="G116" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D116,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D116,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0082</v>
       </c>
-      <c r="H116" s="8" t="str">
+      <c r="H116" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5554,7 +5553,7 @@
         <f t="array" aca="1" ref="G117" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D117,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D117,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0083</v>
       </c>
-      <c r="H117" s="8" t="str">
+      <c r="H117" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5582,7 +5581,7 @@
         <f t="array" aca="1" ref="G118" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D118,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D118,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0084</v>
       </c>
-      <c r="H118" s="8" t="str">
+      <c r="H118" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5610,7 +5609,7 @@
         <f t="array" aca="1" ref="G119" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D119,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D119,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0021</v>
       </c>
-      <c r="H119" s="8" t="str">
+      <c r="H119" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5638,7 +5637,7 @@
         <f t="array" aca="1" ref="G120" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D120,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D120,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0085</v>
       </c>
-      <c r="H120" s="8" t="str">
+      <c r="H120" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5666,7 +5665,7 @@
         <f t="array" aca="1" ref="G121" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D121,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D121,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0040</v>
       </c>
-      <c r="H121" s="8" t="str">
+      <c r="H121" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5694,7 +5693,7 @@
         <f t="array" aca="1" ref="G122" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D122,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D122,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0086</v>
       </c>
-      <c r="H122" s="8" t="str">
+      <c r="H122" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5722,7 +5721,7 @@
         <f t="array" aca="1" ref="G123" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D123,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D123,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0087</v>
       </c>
-      <c r="H123" s="8" t="str">
+      <c r="H123" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5750,7 +5749,7 @@
         <f t="array" aca="1" ref="G124" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D124,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D124,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0088</v>
       </c>
-      <c r="H124" s="8" t="str">
+      <c r="H124" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5778,7 +5777,7 @@
         <f t="array" aca="1" ref="G125" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D125,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D125,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0041</v>
       </c>
-      <c r="H125" s="8" t="str">
+      <c r="H125" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5806,7 +5805,7 @@
         <f t="array" aca="1" ref="G126" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D126,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D126,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0007</v>
       </c>
-      <c r="H126" s="8" t="str">
+      <c r="H126" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5834,7 +5833,7 @@
         <f t="array" aca="1" ref="G127" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D127,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D127,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0082</v>
       </c>
-      <c r="H127" s="8" t="str">
+      <c r="H127" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5862,7 +5861,7 @@
         <f t="array" aca="1" ref="G128" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D128,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D128,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0089</v>
       </c>
-      <c r="H128" s="8" t="str">
+      <c r="H128" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5890,7 +5889,7 @@
         <f t="array" aca="1" ref="G129" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D129,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D129,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0045</v>
       </c>
-      <c r="H129" s="8" t="str">
+      <c r="H129" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5918,7 +5917,7 @@
         <f t="array" aca="1" ref="G130" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D130,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D130,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0072</v>
       </c>
-      <c r="H130" s="8" t="str">
+      <c r="H130" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5946,7 +5945,7 @@
         <f t="array" aca="1" ref="G131" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D131,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D131,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0090</v>
       </c>
-      <c r="H131" s="8" t="str">
+      <c r="H131" t="str">
         <f t="shared" si="1"/>
         <v>STATION</v>
       </c>
@@ -5974,7 +5973,7 @@
         <f t="array" aca="1" ref="G132" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D132,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D132,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0091</v>
       </c>
-      <c r="H132" s="8" t="str">
+      <c r="H132" t="str">
         <f t="shared" ref="H132:H148" si="2">H131</f>
         <v>STATION</v>
       </c>
@@ -6002,7 +6001,7 @@
         <f t="array" aca="1" ref="G133" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D133,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D133,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0091</v>
       </c>
-      <c r="H133" s="8" t="str">
+      <c r="H133" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6030,7 +6029,7 @@
         <f t="array" aca="1" ref="G134" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D134,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D134,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0091</v>
       </c>
-      <c r="H134" s="8" t="str">
+      <c r="H134" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6058,7 +6057,7 @@
         <f t="array" aca="1" ref="G135" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D135,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D135,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0030</v>
       </c>
-      <c r="H135" s="8" t="str">
+      <c r="H135" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6086,7 +6085,7 @@
         <f t="array" aca="1" ref="G136" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D136,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D136,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0092</v>
       </c>
-      <c r="H136" s="8" t="str">
+      <c r="H136" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6114,7 +6113,7 @@
         <f t="array" aca="1" ref="G137" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D137,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D137,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0053</v>
       </c>
-      <c r="H137" s="8" t="str">
+      <c r="H137" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6142,7 +6141,7 @@
         <f t="array" aca="1" ref="G138" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D138,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D138,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0012</v>
       </c>
-      <c r="H138" s="8" t="str">
+      <c r="H138" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6170,7 +6169,7 @@
         <f t="array" aca="1" ref="G139" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D139,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D139,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0093</v>
       </c>
-      <c r="H139" s="8" t="str">
+      <c r="H139" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6198,7 +6197,7 @@
         <f t="array" aca="1" ref="G140" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D140,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D140,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0081</v>
       </c>
-      <c r="H140" s="8" t="str">
+      <c r="H140" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6226,7 +6225,7 @@
         <f t="array" aca="1" ref="G141" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D141,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D141,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0087</v>
       </c>
-      <c r="H141" s="8" t="str">
+      <c r="H141" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6254,7 +6253,7 @@
         <f t="array" aca="1" ref="G142" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D142,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D142,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0027</v>
       </c>
-      <c r="H142" s="8" t="str">
+      <c r="H142" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6282,7 +6281,7 @@
         <f t="array" aca="1" ref="G143" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D143,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D143,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0078</v>
       </c>
-      <c r="H143" s="8" t="str">
+      <c r="H143" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6310,7 +6309,7 @@
         <f t="array" aca="1" ref="G144" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D144,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D144,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0094</v>
       </c>
-      <c r="H144" s="8" t="str">
+      <c r="H144" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6338,7 +6337,7 @@
         <f t="array" aca="1" ref="G145" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D145,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D145,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0095</v>
       </c>
-      <c r="H145" s="8" t="str">
+      <c r="H145" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6366,7 +6365,7 @@
         <f t="array" aca="1" ref="G146" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D146,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D146,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0012</v>
       </c>
-      <c r="H146" s="8" t="str">
+      <c r="H146" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6394,7 +6393,7 @@
         <f t="array" aca="1" ref="G147" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D147,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D147,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0048</v>
       </c>
-      <c r="H147" s="8" t="str">
+      <c r="H147" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
@@ -6422,51 +6421,51 @@
         <f t="array" aca="1" ref="G148" ca="1">"ST"&amp;TEXT(SUMPRODUCT(1/COUNTIF(INDIRECT("$D$2:$D"&amp;(ROW($D$2)+MATCH(D148,$D$2:$D$148,0)-1)),$D$2:INDIRECT("$D"&amp;(ROW($D$2)+MATCH(D148,$D$2:$D$148,0)-1)))),"0000")</f>
         <v>ST0061</v>
       </c>
-      <c r="H148" s="8" t="str">
+      <c r="H148" t="str">
         <f t="shared" si="2"/>
         <v>STATION</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C1:C1048576">
-    <cfRule type="duplicateValues" dxfId="14" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C90">
-    <cfRule type="duplicateValues" dxfId="13" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C84">
-    <cfRule type="duplicateValues" dxfId="12" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="12"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C85">
-    <cfRule type="duplicateValues" dxfId="11" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="11"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C86">
-    <cfRule type="duplicateValues" dxfId="10" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C87">
-    <cfRule type="duplicateValues" dxfId="9" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C88">
-    <cfRule type="duplicateValues" dxfId="8" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C91">
-    <cfRule type="duplicateValues" dxfId="7" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C102">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C108:C111">
-    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="4"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C148">
-    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1">
-    <cfRule type="duplicateValues" dxfId="2" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="14"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D1:D1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -6476,9 +6475,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6626,19 +6628,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2238EE3-A21D-4B6B-9999-BF9A2FCAF6D6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B99169B9-758E-48CB-BCCD-0400850E86A9}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -6662,9 +6660,10 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B99169B9-758E-48CB-BCCD-0400850E86A9}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B2238EE3-A21D-4B6B-9999-BF9A2FCAF6D6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>